<commit_message>
laporan keuangan jaga malam sep2026
</commit_message>
<xml_diff>
--- a/dusun 7/nomor_surat_keluar.xlsx
+++ b/dusun 7/nomor_surat_keluar.xlsx
@@ -1,76 +1,208 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <workbookPr date1904="0"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="60" windowWidth="20055" windowHeight="7950"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3" showHorizontalScroll="1" showVerticalScroll="1"/>
   </bookViews>
   <sheets>
-    <sheet name="surat" sheetId="1" r:id="rId1"/>
-    <sheet name="SK" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="surat" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="SK" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="jenis surat" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="surat_yang_di_keluarkan" sheetId="4" state="visible" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
-  <si>
-    <t>nomor surat</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
+  <si>
+    <t xml:space="preserve">nomor surat</t>
+  </si>
+  <si>
+    <t>tanggal</t>
+  </si>
+  <si>
+    <t>keterangan</t>
+  </si>
+  <si>
+    <t>jenis</t>
   </si>
   <si>
     <t>011/DS.VII/VIII/2026</t>
   </si>
   <si>
-    <t>keterangan</t>
-  </si>
-  <si>
-    <t>tanggal</t>
-  </si>
-  <si>
-    <t>undangan rapat keamanan</t>
+    <t>24-agustus-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">undangan rapat keamanan</t>
+  </si>
+  <si>
+    <t>undangan</t>
+  </si>
+  <si>
+    <t>012/DS.VII/IX/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">surat edaran pemberitahuan jaga malam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">edaran / pemberitahuan</t>
   </si>
   <si>
     <t>01/SK/DS.VII/IX/2026</t>
   </si>
   <si>
-    <t>SK , keamanan</t>
-  </si>
-  <si>
-    <t>24-agustus-2026</t>
-  </si>
-  <si>
     <t>03september2026</t>
   </si>
   <si>
-    <t>012/DS.VII/IX/2026</t>
-  </si>
-  <si>
-    <t>surat edaran pemberitahuan jaga malam</t>
-  </si>
-  <si>
-    <t>jenis</t>
-  </si>
-  <si>
-    <t>undangan</t>
-  </si>
-  <si>
-    <t>edaran / pemberitahuan</t>
+    <t xml:space="preserve">SK , keamanan</t>
+  </si>
+  <si>
+    <t>Kode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jenis Surat</t>
+  </si>
+  <si>
+    <t>UND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surat Undangan</t>
+  </si>
+  <si>
+    <t>KET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surat Keterangan</t>
+  </si>
+  <si>
+    <t>SK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surat Keputusan</t>
+  </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surat Perintah</t>
+  </si>
+  <si>
+    <t>ST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surat Tugas</t>
+  </si>
+  <si>
+    <t>EDR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surat Edaran</t>
+  </si>
+  <si>
+    <t>PMB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surat Pemberitahuan</t>
+  </si>
+  <si>
+    <t>PERM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surat Permohonan</t>
+  </si>
+  <si>
+    <t>PENG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surat Pengantar</t>
+  </si>
+  <si>
+    <t>MOH</t>
+  </si>
+  <si>
+    <t>SRT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surat Biasa</t>
+  </si>
+  <si>
+    <t>BA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Berita Acara</t>
+  </si>
+  <si>
+    <t>NOT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nota Dinas</t>
+  </si>
+  <si>
+    <t>MEMO</t>
+  </si>
+  <si>
+    <t>Memorandum</t>
+  </si>
+  <si>
+    <t>PEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surat Penawaran</t>
+  </si>
+  <si>
+    <t>JAW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surat Jawaban</t>
+  </si>
+  <si>
+    <t>HB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surat Himbauan</t>
+  </si>
+  <si>
+    <t>KEU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">surat Keuangan</t>
+  </si>
+  <si>
+    <t>02/HB/DS.VII/IX/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">himbauan kebersihan</t>
+  </si>
+  <si>
+    <t>03/KEU/DS.VII/X/22026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pembayaran honor jaga malam , bulan september</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="d\-mmm\-yy"/>
+  </numFmts>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10.000000"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -83,30 +215,65 @@
   </fills>
   <borders count="1">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="6">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="43" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="41" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="44" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="42" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="7">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyProtection="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyProtection="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="15" xfId="0" applyNumberFormat="1" applyProtection="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="15" xfId="0" applyNumberFormat="1" applyProtection="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
+    <cellStyle name="Currency" xfId="3" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
+    <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -152,13 +319,13 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Thai" typeface="Angsana New"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
         <a:font script="Gujr" typeface="Shruti"/>
@@ -186,13 +353,13 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Thai" typeface="Cordia New"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
         <a:font script="Gujr" typeface="Shruti"/>
@@ -389,105 +556,521 @@
 </a:theme>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr filterMode="0">
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="27.42578125" customWidth="1"/>
-    <col min="3" max="3" width="39" customWidth="1"/>
-    <col min="4" max="4" width="22.28515625" customWidth="1"/>
+    <col customWidth="1" min="1" max="2" style="0" width="27.420000000000002"/>
+    <col customWidth="1" min="3" max="3" style="0" width="39"/>
+    <col customWidth="1" min="4" max="4" style="0" width="22.289999999999999"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" ht="15">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
+    </row>
+    <row r="5" ht="15">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1">
+        <v>46268</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="1">
-        <v>46268</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D4" t="s">
-        <v>13</v>
-      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.51181102362204689" footer="0.51181102362204689"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr filterMode="0">
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="27.42578125" customWidth="1"/>
-    <col min="3" max="3" width="21.5703125" customWidth="1"/>
+    <col customWidth="1" min="1" max="2" style="0" width="27.420000000000002"/>
+    <col customWidth="1" min="3" max="3" style="0" width="21.57"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" ht="15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" ht="15">
       <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
+        <v>11</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.51181102362204689" footer="0.51181102362204689"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr filterMode="0">
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="2" max="2" style="0" width="22.530000000000001"/>
+    <col customWidth="1" min="3" max="3" style="0" width="17.670000000000002"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" ht="15">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" ht="15">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" ht="15">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" ht="15">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" ht="15">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" ht="15">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" ht="15">
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" ht="15">
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" ht="15">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" ht="15">
+      <c r="A11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" ht="15">
+      <c r="A12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" ht="15">
+      <c r="A13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" ht="15">
+      <c r="A14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" ht="15">
+      <c r="A15" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" ht="15">
+      <c r="A16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17" ht="15">
+      <c r="A17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" ht="15">
+      <c r="A18" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" ht="15">
+      <c r="A19" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.51181102362204689" footer="0.51181102362204689"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr filterMode="0">
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="2" style="0" width="27.420000000000002"/>
+    <col customWidth="1" min="3" max="3" style="0" width="44.140625"/>
+    <col customWidth="1" min="4" max="4" style="0" width="22.289999999999999"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="13.800000000000001">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" ht="13.800000000000001">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" ht="13.800000000000001">
+      <c r="A3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" s="5">
+        <v>46295</v>
+      </c>
+      <c r="C3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" ht="14.25">
+      <c r="A4" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="6">
+        <v>46300</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" ht="13.800000000000001">
+      <c r="B5" s="1"/>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>
+  <pageMargins left="0.78750000000000009" right="0.78750000000000009" top="1.05277777777778" bottom="1.05277777777778" header="0.78750000000000009" footer="0.78750000000000009"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update(nomor_surat_keluar): SK pengurus anggota pengurus masjid
</commit_message>
<xml_diff>
--- a/dusun 7/nomor_surat_keluar.xlsx
+++ b/dusun 7/nomor_surat_keluar.xlsx
@@ -4,11 +4,11 @@
   <workbookPr date1904="0"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3" showHorizontalScroll="1" showVerticalScroll="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1" showHorizontalScroll="1" showVerticalScroll="1"/>
   </bookViews>
   <sheets>
     <sheet name="surat" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="SK" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="SK2026" sheetId="2" state="visible" r:id="rId3"/>
     <sheet name="jenis surat" sheetId="3" state="visible" r:id="rId4"/>
     <sheet name="surat_yang_di_keluarkan" sheetId="4" state="visible" r:id="rId5"/>
   </sheets>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t xml:space="preserve">nomor surat</t>
   </si>
@@ -55,6 +55,9 @@
     <t xml:space="preserve">edaran / pemberitahuan</t>
   </si>
   <si>
+    <t>note</t>
+  </si>
+  <si>
     <t>01/SK/DS.VII/IX/2026</t>
   </si>
   <si>
@@ -64,6 +67,12 @@
     <t xml:space="preserve">SK , keamanan</t>
   </si>
   <si>
+    <t>002/SK/DS.VII/X/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pembentukan pengurus masjid </t>
+  </si>
+  <si>
     <t>Kode</t>
   </si>
   <si>
@@ -181,7 +190,7 @@
     <t xml:space="preserve">himbauan kebersihan</t>
   </si>
   <si>
-    <t>03/KEU/DS.VII/X/22026</t>
+    <t>03/KEU/DS.VII/X/2026</t>
   </si>
   <si>
     <t xml:space="preserve">pembayaran honor jaga malam , bulan september</t>
@@ -232,7 +241,7 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="42" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="0">
       <protection hidden="0" locked="1"/>
     </xf>
@@ -245,10 +254,16 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyProtection="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="0">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" applyProtection="0">
+      <alignment vertical="center"/>
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="15" xfId="0" applyNumberFormat="1" applyProtection="0">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="center"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="15" xfId="0" applyNumberFormat="1" applyProtection="0">
@@ -793,10 +808,12 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="2" style="0" width="27.420000000000002"/>
-    <col customWidth="1" min="3" max="3" style="0" width="21.57"/>
+    <col customWidth="1" min="3" max="3" style="0" width="31.140625"/>
+    <col customWidth="1" min="4" max="4" width="14.421875"/>
+    <col customWidth="1" min="5" max="5" width="63.140625"/>
   </cols>
   <sheetData>
     <row r="1" ht="15">
@@ -809,17 +826,35 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="2" ht="15">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>13</v>
-      </c>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" ht="57">
+      <c r="A3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="5">
+        <v>46309</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>
@@ -843,154 +878,154 @@
   <sheetData>
     <row r="1" ht="15">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" ht="15">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" ht="15">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" ht="15">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" ht="15">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" ht="15">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" ht="15">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" ht="15">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" ht="15">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" ht="15">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" ht="15">
       <c r="A11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" t="s">
         <v>34</v>
-      </c>
-      <c r="B11" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="12" ht="15">
       <c r="A12" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B12" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" ht="15">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" ht="15">
       <c r="A14" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B14" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" ht="15">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" ht="15">
       <c r="A16" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" ht="15">
       <c r="A17" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B17" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" ht="15">
       <c r="A18" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B18" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" ht="15">
       <c r="A19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1027,42 +1062,47 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="2" ht="13.800000000000001">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" ht="13.800000000000001">
       <c r="A3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B3" s="5">
+        <v>54</v>
+      </c>
+      <c r="B3" s="7">
         <v>46295</v>
       </c>
       <c r="C3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" ht="14.25">
-      <c r="A4" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B4" s="6">
+      <c r="A4" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="7">
         <v>46300</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>54</v>
+      <c r="C4" s="2" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="5" ht="13.800000000000001">
+      <c r="A5" s="2"/>
       <c r="B5" s="1"/>
+      <c r="C5" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>

</xml_diff>